<commit_message>
Stock import template: one example row only
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01G9w5PhNoNDSSXobyjzq7rs
</commit_message>
<xml_diff>
--- a/react-app/public/stock-holdings-sample.xlsx
+++ b/react-app/public/stock-holdings-sample.xlsx
@@ -448,7 +448,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C7"/>
+  <dimension ref="A1:C2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
@@ -484,71 +484,6 @@
       </c>
       <c r="C2" s="4" t="n">
         <v>2450.5</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="2" t="inlineStr">
-        <is>
-          <t>INFY</t>
-        </is>
-      </c>
-      <c r="B3" s="3" t="n">
-        <v>25</v>
-      </c>
-      <c r="C3" s="4" t="n">
-        <v>1520</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="2" t="inlineStr">
-        <is>
-          <t>HDFCBANK</t>
-        </is>
-      </c>
-      <c r="B4" s="3" t="n">
-        <v>15</v>
-      </c>
-      <c r="C4" s="4" t="n">
-        <v>1610.25</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="2" t="inlineStr">
-        <is>
-          <t>TCS</t>
-        </is>
-      </c>
-      <c r="B5" s="3" t="n">
-        <v>5</v>
-      </c>
-      <c r="C5" s="4" t="n">
-        <v>3890</v>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="2" t="inlineStr">
-        <is>
-          <t>NIFTYBEES</t>
-        </is>
-      </c>
-      <c r="B6" s="3" t="n">
-        <v>100</v>
-      </c>
-      <c r="C6" s="4" t="n">
-        <v>265.4</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="2" t="inlineStr">
-        <is>
-          <t>GOLDBEES</t>
-        </is>
-      </c>
-      <c r="B7" s="3" t="n">
-        <v>200</v>
-      </c>
-      <c r="C7" s="4" t="n">
-        <v>58.75</v>
       </c>
     </row>
   </sheetData>
@@ -606,7 +541,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Delete the example rows and add your own. Only the Holdings sheet is read.</t>
+          <t>Replace the example row with your own, one stock per row. Only the Holdings sheet is read.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Stock search and import for any market: US stocks/ETFs list in search, BSE-only stocks tagged BSE, any Google Finance symbol (LON:VOD, BOM:517015); import template with optional Currency and Buy date columns (old 3-column files unchanged); buy/sell forms work in any currency
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01G9w5PhNoNDSSXobyjzq7rs
</commit_message>
<xml_diff>
--- a/react-app/public/stock-holdings-sample.xlsx
+++ b/react-app/public/stock-holdings-sample.xlsx
@@ -17,7 +17,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
+  </numFmts>
   <fonts count="3">
     <font>
       <name val="Calibri"/>
@@ -48,7 +50,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -56,32 +58,14 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color rgb="00D0D5DD"/>
-      </left>
-      <right style="thin">
-        <color rgb="00D0D5DD"/>
-      </right>
-      <top style="thin">
-        <color rgb="00D0D5DD"/>
-      </top>
-      <bottom style="thin">
-        <color rgb="00D0D5DD"/>
-      </bottom>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="4" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -448,12 +432,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C2"/>
+  <dimension ref="A1:E4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="16" customWidth="1" min="1" max="1"/>
-    <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="11" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="11" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -472,19 +458,70 @@
           <t>Avg Price</t>
         </is>
       </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Currency</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Buy date</t>
+        </is>
+      </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr">
+      <c r="A2" t="inlineStr">
         <is>
           <t>RELIANCE</t>
         </is>
       </c>
-      <c r="B2" s="3" t="n">
+      <c r="B2" t="n">
         <v>10</v>
       </c>
-      <c r="C2" s="4" t="n">
+      <c r="C2" t="n">
         <v>2450.5</v>
       </c>
+      <c r="E2" s="2" t="n"/>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>AAPL</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>5</v>
+      </c>
+      <c r="C3" t="n">
+        <v>182.5</v>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="n">
+        <v>45366</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>VOO</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>3</v>
+      </c>
+      <c r="C4" t="n">
+        <v>455</v>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -497,65 +534,85 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A8"/>
+  <dimension ref="A1:A12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="90" customWidth="1" min="1" max="1"/>
+    <col width="120" customWidth="1" min="1" max="1"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="5" t="inlineStr">
+      <c r="A1" s="3" t="inlineStr">
         <is>
           <t>How to fill this file</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>1. Symbol: the NSE symbol, e.g. RELIANCE, INFY, NIFTYBEES (ETFs work too).</t>
-        </is>
-      </c>
+      <c r="A2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2. Quantity: number of shares you hold.</t>
+          <t>1. Symbol: the NSE symbol, e.g. RELIANCE, INFY, NIFTYBEES (ETFs work too). A BSE-only stock: its BSE code as BOM:517015.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>3. Avg Price: your average buy price per share.</t>
+          <t>2. Quantity: number of shares you hold.</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Keep the first row (Symbol, Quantity, Avg Price) as it is. One stock per row.</t>
+          <t>3. Avg Price: your average buy price per share.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Replace the example row with your own, one stock per row. Only the Holdings sheet is read.</t>
+          <t>4. Currency (optional): leave blank for Indian stocks (₹). For US stocks write USD and the price in $, e.g. AAPL · 5 · 182.50 · USD.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Then in the app: Stocks &gt; Import &gt; choose this file.</t>
+          <t xml:space="preserve">   Other markets: write the symbol as on Google Finance (LON:VOD, TYO:7203) and the price in that market's currency.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Live price, value and P&amp;L come from Google Finance automatically.</t>
+          <t>5. Buy date (optional): the price is turned into ₹ with that day's rate. Blank = the date you pick in the app.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr"/>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Keep the first row as it is. One stock per row. Replace the example rows with your own. Only the Holdings sheet is read.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Old files with just Symbol, Quantity, Avg Price still work.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Then in the app: Stocks &gt; Import &gt; choose this file. Live price, value and P&amp;L come from Google Finance automatically.</t>
         </is>
       </c>
     </row>

</xml_diff>